<commit_message>
Build size updated to 15mb
</commit_message>
<xml_diff>
--- a/documents/Task.xlsx
+++ b/documents/Task.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
   <si>
     <t>Sr.no</t>
   </si>
@@ -261,7 +261,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">(feature/login) :- Puch new commited code of local to remote repo's specifice branch.
-Command to deploy Angular application to GitHub
+Command to deploy Angular application to GitHub (Run in cmd)
     - </t>
     </r>
     <r>
@@ -305,8 +305,20 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>(after every puch) :- build your Angular application and deploy it to GitHub
-                        Pages, while telling Angular that the application will be hosted inside the /RentalManagementSystem/ path.</t>
+      <t xml:space="preserve">(after every puch) :- build your Angular application and deploy it to GitHub
+                        Pages, while telling Angular that the application will be hosted inside the /RentalManagementSystem/ path.
+    - command - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ng deploy --base-href=/RentalManagementSystem/</t>
     </r>
   </si>
 </sst>
@@ -873,7 +885,7 @@
       </c>
       <c r="F9" s="14"/>
     </row>
-    <row r="10" spans="1:6" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="174" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -905,7 +917,9 @@
       <c r="E11" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="14"/>
+      <c r="F11" s="14" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="1:6" ht="116" x14ac:dyDescent="0.35">
       <c r="A12" s="6">

</xml_diff>

<commit_message>
Added - Billing feature and animations
</commit_message>
<xml_diff>
--- a/documents/Task.xlsx
+++ b/documents/Task.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
   <si>
     <t>Sr.no</t>
   </si>
@@ -328,6 +328,62 @@
     - Add Tenant details page.
     - Add Create Tenant button to the tenant page
     - Add Create Tenant page</t>
+  </si>
+  <si>
+    <t>Pages - 
+     - Create page called bashboard where all the info realated to the owner will be disblayed.
+     - Added dashborad.model.ts in core/models
+     - Added dashboard.service.ts in core/service
+     - Added test data in core/test-data and updated index in core/test-data
+     - Added Overview page in pages/dashboard
+     - Added animation to the overview page</t>
+  </si>
+  <si>
+    <r>
+      <t>Pages - 
+    - Enhanced UI of Nave bar for android and windows.
+    - Add amination for the porperty, tenant, side bar and login page.
+    - Update font to "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Plus Jakarta Sans</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>".
+    - Create a SnackBar service for login page.
+    - Added animation to the property's card info.
+    - Added animation to the tenant's card for android and tablet.</t>
+    </r>
+  </si>
+  <si>
+    <t>Pages - 
+    - Update the module of Billing(from scratch).
+    - Added billing-generated and billing-pending tab to Billing module.
+    - Added bill-details mdoule.
+    - Added generate-bill form to generate bill.
+    - Added generate-this-months-bill button and view-this-months-bill button to the room-details card.</t>
+  </si>
+  <si>
+    <t>Pages - 
+    - Updated alignment to the billing section.
+    - Added animation to billing section.
+    - Updated minor variable of billing section. 
+    - Improve the animation of side bar in windows screen.</t>
   </si>
 </sst>
 </file>
@@ -371,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -405,6 +461,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -763,16 +834,16 @@
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="19">
         <v>46248</v>
       </c>
-      <c r="D2" s="16">
+      <c r="D2" s="21">
         <v>46250</v>
       </c>
-      <c r="E2" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="13" t="s">
+      <c r="E2" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="18" t="s">
         <v>15</v>
       </c>
     </row>
@@ -783,10 +854,10 @@
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
     </row>
     <row r="4" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A4" s="6">
@@ -804,7 +875,7 @@
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="13"/>
+      <c r="F4" s="18"/>
     </row>
     <row r="5" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A5" s="6">
@@ -822,7 +893,7 @@
       <c r="E5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="13"/>
+      <c r="F5" s="18"/>
     </row>
     <row r="6" spans="1:6" ht="116" x14ac:dyDescent="0.35">
       <c r="A6" s="6">
@@ -840,7 +911,7 @@
       <c r="E6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="13"/>
+      <c r="F6" s="18"/>
     </row>
     <row r="7" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A7" s="6">
@@ -858,7 +929,7 @@
       <c r="E7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="13"/>
+      <c r="F7" s="18"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
@@ -876,7 +947,7 @@
       <c r="E8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="13"/>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="6">
@@ -894,7 +965,7 @@
       <c r="E9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="13"/>
+      <c r="F9" s="18"/>
     </row>
     <row r="10" spans="1:6" ht="174" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
@@ -912,7 +983,7 @@
       <c r="E10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F10" s="13"/>
+      <c r="F10" s="18"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="6"/>
@@ -928,7 +999,7 @@
       <c r="E11" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="18" t="s">
         <v>15</v>
       </c>
     </row>
@@ -948,7 +1019,7 @@
       <c r="E12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="13"/>
+      <c r="F12" s="18"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
@@ -966,7 +1037,7 @@
       <c r="E13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F13" s="13"/>
+      <c r="F13" s="18"/>
     </row>
     <row r="14" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
@@ -984,7 +1055,7 @@
       <c r="E14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F14" s="13"/>
+      <c r="F14" s="18"/>
     </row>
     <row r="15" spans="1:6" s="11" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
@@ -1002,7 +1073,7 @@
       <c r="E15" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F15" s="13"/>
+      <c r="F15" s="18"/>
     </row>
     <row r="16" spans="1:6" s="11" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="6"/>
@@ -1016,7 +1087,7 @@
       <c r="E16" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="13"/>
+      <c r="F16" s="18"/>
     </row>
     <row r="17" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
@@ -1034,7 +1105,7 @@
       <c r="E17" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F17" s="13"/>
+      <c r="F17" s="18"/>
     </row>
     <row r="18" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
@@ -1056,34 +1127,70 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="6"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
+    <row r="19" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="6">
+        <v>16</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="13">
+        <v>46266</v>
+      </c>
+      <c r="D19" s="14">
+        <v>46268</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>8</v>
+      </c>
       <c r="F19" s="10"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="6"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
+    <row r="20" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="6">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="15">
+        <v>46268</v>
+      </c>
+      <c r="D20" s="15">
+        <v>46269</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>8</v>
+      </c>
       <c r="F20" s="10"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="6"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
+    <row r="21" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+      <c r="A21" s="6">
+        <v>18</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="16">
+        <v>46269</v>
+      </c>
+      <c r="D21" s="17">
+        <v>46271</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>8</v>
+      </c>
       <c r="F21" s="10"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="6"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="3"/>
+    <row r="22" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="6">
+        <v>19</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="17">
+        <v>46271</v>
+      </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>

</xml_diff>

<commit_message>
Animation removed of side bar for android
</commit_message>
<xml_diff>
--- a/documents/Task.xlsx
+++ b/documents/Task.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="31">
   <si>
     <t>Sr.no</t>
   </si>
@@ -384,6 +384,9 @@
     - Added animation to billing section.
     - Updated minor variable of billing section. 
     - Improve the animation of side bar in windows screen.</t>
+  </si>
+  <si>
+    <t>animation removed of side bar for android</t>
   </si>
 </sst>
 </file>
@@ -427,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -461,6 +464,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -834,16 +840,16 @@
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="19">
+      <c r="C2" s="20">
         <v>46248</v>
       </c>
-      <c r="D2" s="21">
+      <c r="D2" s="22">
         <v>46250</v>
       </c>
-      <c r="E2" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="18" t="s">
+      <c r="E2" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="19" t="s">
         <v>15</v>
       </c>
     </row>
@@ -854,10 +860,10 @@
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
     </row>
     <row r="4" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A4" s="6">
@@ -875,7 +881,7 @@
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="18"/>
+      <c r="F4" s="19"/>
     </row>
     <row r="5" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A5" s="6">
@@ -893,7 +899,7 @@
       <c r="E5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="18"/>
+      <c r="F5" s="19"/>
     </row>
     <row r="6" spans="1:6" ht="116" x14ac:dyDescent="0.35">
       <c r="A6" s="6">
@@ -911,7 +917,7 @@
       <c r="E6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="18"/>
+      <c r="F6" s="19"/>
     </row>
     <row r="7" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A7" s="6">
@@ -929,7 +935,7 @@
       <c r="E7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="18"/>
+      <c r="F7" s="19"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
@@ -947,7 +953,7 @@
       <c r="E8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="18"/>
+      <c r="F8" s="19"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="6">
@@ -965,7 +971,7 @@
       <c r="E9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="18"/>
+      <c r="F9" s="19"/>
     </row>
     <row r="10" spans="1:6" ht="174" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
@@ -983,7 +989,7 @@
       <c r="E10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F10" s="18"/>
+      <c r="F10" s="19"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="6"/>
@@ -999,7 +1005,7 @@
       <c r="E11" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1019,7 +1025,7 @@
       <c r="E12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="18"/>
+      <c r="F12" s="19"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
@@ -1037,7 +1043,7 @@
       <c r="E13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F13" s="18"/>
+      <c r="F13" s="19"/>
     </row>
     <row r="14" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
@@ -1055,7 +1061,7 @@
       <c r="E14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F14" s="18"/>
+      <c r="F14" s="19"/>
     </row>
     <row r="15" spans="1:6" s="11" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
@@ -1073,7 +1079,7 @@
       <c r="E15" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F15" s="18"/>
+      <c r="F15" s="19"/>
     </row>
     <row r="16" spans="1:6" s="11" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="6"/>
@@ -1087,7 +1093,7 @@
       <c r="E16" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="18"/>
+      <c r="F16" s="19"/>
     </row>
     <row r="17" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
@@ -1105,7 +1111,7 @@
       <c r="E17" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F17" s="18"/>
+      <c r="F17" s="19"/>
     </row>
     <row r="18" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
@@ -1143,7 +1149,9 @@
       <c r="E19" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F19" s="10"/>
+      <c r="F19" s="19" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A20" s="6">
@@ -1161,7 +1169,7 @@
       <c r="E20" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F20" s="10"/>
+      <c r="F20" s="19"/>
     </row>
     <row r="21" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A21" s="6">
@@ -1179,7 +1187,7 @@
       <c r="E21" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F21" s="10"/>
+      <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A22" s="6">
@@ -1191,17 +1199,31 @@
       <c r="C22" s="17">
         <v>46271</v>
       </c>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
+      <c r="D22" s="18">
+        <v>46272</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="19"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="6"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="A23" s="6">
+        <v>20</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="18">
+        <v>46271</v>
+      </c>
+      <c r="D23" s="18">
+        <v>46271</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="19"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="6"/>
@@ -1276,7 +1298,8 @@
       <c r="F32" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="F19:F23"/>
     <mergeCell ref="F11:F17"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>

</xml_diff>